<commit_message>
vendor risk profiling added
</commit_message>
<xml_diff>
--- a/data/seed/responses/shree_balaji/SBP_Quotation_0914.xlsx
+++ b/data/seed/responses/shree_balaji/SBP_Quotation_0914.xlsx
@@ -1387,7 +1387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1478,6 +1478,42 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Turnover (FY 2025-26)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Rs. 85 crore</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Established</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Credit rating</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CRISIL BBB+ / Stable</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>